<commit_message>
Add new functionality and tests for account management and permissions
- Introduced `initialize-accounts.ts` script to prepare account schema in the dashboard.
- Added `permissions.test.ts` to validate user permissions and authentication processes.
- Included new Excel files for app functionality testing and dummy data export.
- Updated existing `firtech_dashboard.xlsx` to reflect changes in account management.
- Ensured that guest users have read-only access and contributors are restricted by department.
- Implemented tests for user authentication and permissions round-trip, ensuring password hashes are omitted from audit logs.
</commit_message>
<xml_diff>
--- a/fir-tech-intelligent-automation-hub/public/firtech_dashboard.xlsx
+++ b/fir-tech-intelligent-automation-hub/public/firtech_dashboard.xlsx
@@ -1,45 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_1A07B81E5C7F59B972A77098AC8B625CE9FB1C2C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67C164A8-F1EE-43B6-A09B-C9F1B957AA6E}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12000" windowHeight="24000"/>
   </bookViews>
   <sheets>
-    <sheet name="Settings" sheetId="1" r:id="rId1"/>
-    <sheet name="Departments" sheetId="2" r:id="rId2"/>
-    <sheet name="People" sheetId="3" r:id="rId3"/>
-    <sheet name="Memberships" sheetId="4" r:id="rId4"/>
-    <sheet name="Requirements" sheetId="5" r:id="rId5"/>
-    <sheet name="Training" sheetId="6" r:id="rId6"/>
-    <sheet name="Opportunities" sheetId="7" r:id="rId7"/>
-    <sheet name="Engagements" sheetId="8" r:id="rId8"/>
-    <sheet name="Audit" sheetId="9" r:id="rId9"/>
+    <sheet sheetId="1" name="Settings" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Departments" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="People" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Memberships" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Requirements" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Training" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Opportunities" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Engagements" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Audit" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Users" state="visible" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="191028" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="252">
   <si>
     <t>Setting</t>
   </si>
@@ -765,19 +749,52 @@
   </si>
   <si>
     <t>Seeded from supplied specification</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>PasswordHash</t>
+  </si>
+  <si>
+    <t>Departments</t>
+  </si>
+  <si>
+    <t>ExportReports</t>
+  </si>
+  <si>
+    <t>ManagePathways</t>
+  </si>
+  <si>
+    <t>ManageUsers</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>pbkdf2$b24bcfdd-82da-48be-9433-fcd80da609fa$0bfe3132c6ecef76176641d961b45f0e32ee34d11ab66f42487829b72e24017b</t>
+  </si>
+  <si>
+    <t>Administrator</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -800,14 +817,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1140,11 +1158,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1152,7 +1170,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1160,7 +1178,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1168,7 +1186,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1176,7 +1194,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1184,7 +1202,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1192,7 +1210,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1200,7 +1218,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1208,7 +1226,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1218,18 +1236,81 @@
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:B9" numberStoredAsText="1"/>
-  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="8" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -1258,7 +1339,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1287,7 +1368,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1316,7 +1397,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -1345,7 +1426,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -1374,7 +1455,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1403,7 +1484,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>41</v>
       </c>
@@ -1432,7 +1513,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1463,18 +1544,15 @@
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:I8" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>46</v>
       </c>
@@ -1506,7 +1584,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>55</v>
       </c>
@@ -1538,7 +1616,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>59</v>
       </c>
@@ -1570,7 +1648,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1602,7 +1680,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>66</v>
       </c>
@@ -1634,7 +1712,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>69</v>
       </c>
@@ -1666,7 +1744,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>71</v>
       </c>
@@ -1698,7 +1776,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -1730,7 +1808,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>75</v>
       </c>
@@ -1762,7 +1840,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>77</v>
       </c>
@@ -1794,7 +1872,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>80</v>
       </c>
@@ -1826,7 +1904,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>82</v>
       </c>
@@ -1860,18 +1938,15 @@
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:J12" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -1894,7 +1969,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>89</v>
       </c>
@@ -1917,7 +1992,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>91</v>
       </c>
@@ -1940,7 +2015,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>92</v>
       </c>
@@ -1963,7 +2038,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>93</v>
       </c>
@@ -1986,7 +2061,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>94</v>
       </c>
@@ -2011,18 +2086,15 @@
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:G6" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>95</v>
       </c>
@@ -2060,7 +2132,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>104</v>
       </c>
@@ -2098,7 +2170,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>110</v>
       </c>
@@ -2136,7 +2208,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>113</v>
       </c>
@@ -2174,7 +2246,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>117</v>
       </c>
@@ -2212,7 +2284,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>119</v>
       </c>
@@ -2250,7 +2322,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>121</v>
       </c>
@@ -2288,7 +2360,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>123</v>
       </c>
@@ -2326,7 +2398,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>125</v>
       </c>
@@ -2364,7 +2436,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>128</v>
       </c>
@@ -2402,7 +2474,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>130</v>
       </c>
@@ -2440,7 +2512,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>134</v>
       </c>
@@ -2478,7 +2550,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>138</v>
       </c>
@@ -2516,7 +2588,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>140</v>
       </c>
@@ -2554,7 +2626,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>142</v>
       </c>
@@ -2592,7 +2664,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>144</v>
       </c>
@@ -2630,7 +2702,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>145</v>
       </c>
@@ -2670,18 +2742,15 @@
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:L17" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>147</v>
       </c>
@@ -2716,7 +2785,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>151</v>
       </c>
@@ -2751,7 +2820,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>155</v>
       </c>
@@ -2786,7 +2855,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>158</v>
       </c>
@@ -2821,7 +2890,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>163</v>
       </c>
@@ -2858,18 +2927,15 @@
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:K5" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>166</v>
       </c>
@@ -2913,7 +2979,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>178</v>
       </c>
@@ -2936,7 +3002,7 @@
         <v>850000</v>
       </c>
       <c r="H2">
-        <v>0.55000000000000004</v>
+        <v>0.55</v>
       </c>
       <c r="I2">
         <v>467500</v>
@@ -2957,7 +3023,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>185</v>
       </c>
@@ -3001,7 +3067,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>192</v>
       </c>
@@ -3045,7 +3111,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>199</v>
       </c>
@@ -3091,18 +3157,15 @@
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:N5" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>206</v>
       </c>
@@ -3140,7 +3203,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>214</v>
       </c>
@@ -3178,7 +3241,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>221</v>
       </c>
@@ -3218,18 +3281,15 @@
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:L3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>226</v>
       </c>
@@ -3258,7 +3318,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>234</v>
       </c>
@@ -3289,8 +3349,5 @@
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:I2" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Update report metrics and enhance workbook functionality
- Renamed "UiPath revenue (USD)" to "Recorded revenue (USD)" in reports.
- Improved CSV export functionality by ensuring headers are escaped correctly.
- Added undo functionality for workbook mutations, preserving audit history.
- Enhanced WorkbookProvider to manage download confirmations and state.
- Created new tests for delivery gate processes, ensuring stable IDs and audit preservation.
- Implemented report export tests to validate CSV and Excel outputs.
- Added missing worksheets to the firtech_dashboard.xlsx file.
- Updated build and QA documentation for clarity and completeness.
</commit_message>
<xml_diff>
--- a/fir-tech-intelligent-automation-hub/public/firtech_dashboard.xlsx
+++ b/fir-tech-intelligent-automation-hub/public/firtech_dashboard.xlsx
@@ -17,13 +17,16 @@
     <sheet sheetId="8" name="Engagements" state="visible" r:id="rId11"/>
     <sheet sheetId="9" name="Audit" state="visible" r:id="rId12"/>
     <sheet sheetId="10" name="Users" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="Leads" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="Revenue" state="visible" r:id="rId15"/>
+    <sheet sheetId="13" name="Certifications" state="visible" r:id="rId16"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="275">
   <si>
     <t>Setting</t>
   </si>
@@ -779,13 +782,82 @@
   </si>
   <si>
     <t>*</t>
+  </si>
+  <si>
+    <t>LeadId</t>
+  </si>
+  <si>
+    <t>DepartmentId</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>CreatedDate</t>
+  </si>
+  <si>
+    <t>ReportingCurrency</t>
+  </si>
+  <si>
+    <t>ConvertedAmount</t>
+  </si>
+  <si>
+    <t>ExchangeRate</t>
+  </si>
+  <si>
+    <t>ExchangeRateDate</t>
+  </si>
+  <si>
+    <t>ExchangeRateSource</t>
+  </si>
+  <si>
+    <t>RevenueId</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>OwnerDepartmentId</t>
+  </si>
+  <si>
+    <t>LeadOriginDepartmentId</t>
+  </si>
+  <si>
+    <t>InfluencingDepartmentId</t>
+  </si>
+  <si>
+    <t>DeliveringDepartmentId</t>
+  </si>
+  <si>
+    <t>RecognizedDate</t>
+  </si>
+  <si>
+    <t>CertificationId</t>
+  </si>
+  <si>
+    <t>PersonId</t>
+  </si>
+  <si>
+    <t>CertName</t>
+  </si>
+  <si>
+    <t>IssueDate</t>
+  </si>
+  <si>
+    <t>ExpiryDate</t>
+  </si>
+  <si>
+    <t>UiPathCertCode</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -796,13 +868,22 @@
     <font>
       <b/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF216689"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -817,9 +898,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1301,6 +1383,165 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="14" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="15" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="8" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>